<commit_message>
Plan del sprint: estado de las tareas de codigo segun la revision del 23-24/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etica docs/Plan_Sprint_SIS321_MedicalSys.xlsx
+++ b/etica docs/Plan_Sprint_SIS321_MedicalSys.xlsx
@@ -26,10 +26,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="ddd dd/mm"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -224,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -249,7 +248,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -309,7 +308,7 @@
     <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -343,6 +342,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -949,7 +954,7 @@
         <f>COUNTIF(Tareas!$D$5:$D$77,A15)</f>
         <v/>
       </c>
-      <c r="E15" s="14">
+      <c r="E15" s="48">
         <f>SUMIF(Tareas!$D$5:$D$77,A15,Tareas!$M$5:$M$77)</f>
         <v/>
       </c>
@@ -982,7 +987,7 @@
         <f>COUNTIF(Tareas!$D$5:$D$77,A16)</f>
         <v/>
       </c>
-      <c r="E16" s="14">
+      <c r="E16" s="48">
         <f>SUMIF(Tareas!$D$5:$D$77,A16,Tareas!$M$5:$M$77)</f>
         <v/>
       </c>
@@ -1015,7 +1020,7 @@
         <f>COUNTIF(Tareas!$D$5:$D$77,A17)</f>
         <v/>
       </c>
-      <c r="E17" s="14">
+      <c r="E17" s="48">
         <f>SUMIF(Tareas!$D$5:$D$77,A17,Tareas!$M$5:$M$77)</f>
         <v/>
       </c>
@@ -1048,7 +1053,7 @@
         <f>COUNTIF(Tareas!$D$5:$D$77,A18)</f>
         <v/>
       </c>
-      <c r="E18" s="14">
+      <c r="E18" s="48">
         <f>SUMIF(Tareas!$D$5:$D$77,A18,Tareas!$M$5:$M$77)</f>
         <v/>
       </c>
@@ -1081,7 +1086,7 @@
         <f>COUNTIF(Tareas!$D$5:$D$77,A19)</f>
         <v/>
       </c>
-      <c r="E19" s="14">
+      <c r="E19" s="48">
         <f>SUMIF(Tareas!$D$5:$D$77,A19,Tareas!$M$5:$M$77)</f>
         <v/>
       </c>
@@ -1114,7 +1119,7 @@
         <f>COUNTIF(Tareas!$D$5:$D$77,A20)</f>
         <v/>
       </c>
-      <c r="E20" s="14">
+      <c r="E20" s="48">
         <f>SUMIF(Tareas!$D$5:$D$77,A20,Tareas!$M$5:$M$77)</f>
         <v/>
       </c>
@@ -1788,8 +1793,8 @@
     <mergeCell ref="B43:H43"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B50:G50"/>
+    <mergeCell ref="B42:H42"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="B42:H42"/>
     <mergeCell ref="C34:H34"/>
     <mergeCell ref="B60:H60"/>
     <mergeCell ref="C30:H30"/>
@@ -2034,7 +2039,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="M5" s="48" t="n">
         <v>1</v>
       </c>
       <c r="N5" s="12" t="inlineStr">
@@ -2128,7 +2133,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="M6" s="48" t="n">
         <v>0.5</v>
       </c>
       <c r="N6" s="12" t="inlineStr">
@@ -2222,7 +2227,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M7" s="14" t="n">
+      <c r="M7" s="48" t="n">
         <v>2</v>
       </c>
       <c r="N7" s="12" t="inlineStr">
@@ -2252,10 +2257,15 @@
       </c>
       <c r="S7" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T7" s="30" t="inlineStr"/>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="T7" s="30" t="inlineStr">
+        <is>
+          <t>[Corregido 24/10] CI/CD del backend reactivado por Alvaro (push a main despliega) y del frontend reactivado. En producción, GATEWAY_ALLOWED_ORIGINS debe incluir https://medicalsys.los5furiosos.cloud o el login falla por CORS.
+[Revisión de código 23/10] Merge de todas las ramas a develop y main hecho (4d0f660), con pruebas unitarias y e2e en verde. Falta: tag v-seg-1, SHA256SUMS de la entrega y despliegue en el enlace público.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="25" t="inlineStr">
@@ -2316,7 +2326,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M8" s="14" t="n">
+      <c r="M8" s="48" t="n">
         <v>2</v>
       </c>
       <c r="N8" s="12" t="inlineStr">
@@ -2410,7 +2420,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M9" s="14" t="n">
+      <c r="M9" s="48" t="n">
         <v>4</v>
       </c>
       <c r="N9" s="12" t="inlineStr">
@@ -2440,10 +2450,14 @@
       </c>
       <c r="S9" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T9" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T9" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] Keycloak 26.7.5 con el realm medicalsys importado; smoke-token.sh en verde. Decisión GO.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="25" t="inlineStr">
@@ -2504,7 +2518,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M10" s="14" t="n">
+      <c r="M10" s="48" t="n">
         <v>2</v>
       </c>
       <c r="N10" s="12" t="inlineStr">
@@ -2534,10 +2548,14 @@
       </c>
       <c r="S10" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T10" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T10" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] policy-check.sh en verde: 9 reglas, histórico de 5, Argon2id y bloqueo permanente al 3er intento. Realm versionado en infra/keycloak.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="25" t="inlineStr">
@@ -2598,7 +2616,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M11" s="14" t="n">
+      <c r="M11" s="48" t="n">
         <v>5</v>
       </c>
       <c r="N11" s="12" t="inlineStr">
@@ -2628,10 +2646,14 @@
       </c>
       <c r="S11" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T11" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T11" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] Login delegado a Keycloak: 200, 401 genérico, 423 bloqueada y 403 PASSWORD_CHANGE_REQUIRED verificados (login-keycloak.sh y e2e.sh). Tests de AuthService.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="25" t="inlineStr">
@@ -2692,7 +2714,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M12" s="14" t="n">
+      <c r="M12" s="48" t="n">
         <v>5</v>
       </c>
       <c r="N12" s="12" t="inlineStr">
@@ -2722,10 +2744,14 @@
       </c>
       <c r="S12" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T12" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T12" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] Alta, modificación y baja sincronizadas con Keycloak (la baja deshabilita, no borra). User ID MS-AA-NNNNN (migración V7) con tests.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="25" t="inlineStr">
@@ -2786,7 +2812,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M13" s="14" t="n">
+      <c r="M13" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N13" s="12" t="inlineStr">
@@ -2816,10 +2842,14 @@
       </c>
       <c r="S13" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T13" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T13" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] Bloqueo al 3er intento → desbloqueo → reinicio con temporal → cambio forzado → reutilizar anterior rechazado (desbloqueo-reinicio.sh).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="25" t="inlineStr">
@@ -2880,7 +2910,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M14" s="14" t="n">
+      <c r="M14" s="48" t="n">
         <v>4</v>
       </c>
       <c r="N14" s="12" t="inlineStr">
@@ -2910,10 +2940,14 @@
       </c>
       <c r="S14" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T14" s="30" t="inlineStr"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="T14" s="30" t="inlineStr">
+        <is>
+          <t>[Frontend 24/10] Integrada en main/develop del frontend (sins-59). Verificado en el navegador contra el backend: lista con User ID y estado de las 28 cuentas; los botones de alta, edición, baja, desbloqueo y reinicio llaman a los endpoints correctos; 103 tests del frontend en verde. Falta recorrer la demo completa en vivo (alta → temporal → desbloqueo → reinicio).</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="25" t="inlineStr">
@@ -2974,7 +3008,7 @@
           <t>Baja</t>
         </is>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="M15" s="48" t="n">
         <v>6</v>
       </c>
       <c r="N15" s="12" t="inlineStr">
@@ -3004,10 +3038,14 @@
       </c>
       <c r="S15" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T15" s="30" t="inlineStr"/>
+          <t>Cancelada</t>
+        </is>
+      </c>
+      <c r="T15" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] IAM-01 dio GO: el plan B no se activa.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="25" t="inlineStr">
@@ -3068,7 +3106,7 @@
           <t>Baja</t>
         </is>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="M16" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N16" s="12" t="inlineStr">
@@ -3101,7 +3139,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="T16" s="30" t="inlineStr"/>
+      <c r="T16" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] Opcional. El realm no tiene WebAuthn/passkeys configurado.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="25" t="inlineStr">
@@ -3162,7 +3204,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M17" s="14" t="n">
+      <c r="M17" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N17" s="12" t="inlineStr">
@@ -3256,7 +3298,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M18" s="14" t="n">
+      <c r="M18" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N18" s="12" t="inlineStr">
@@ -3286,10 +3328,14 @@
       </c>
       <c r="S18" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T18" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T18" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] GET /api/v1/identity/permissions devuelve 169 permisos; los 252 endpoints coinciden con la matriz (scripts/ci/check_permissions.py).</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="25" t="inlineStr">
@@ -3350,7 +3396,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M19" s="14" t="n">
+      <c r="M19" s="48" t="n">
         <v>5</v>
       </c>
       <c r="N19" s="12" t="inlineStr">
@@ -3380,10 +3426,15 @@
       </c>
       <c r="S19" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T19" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T19" s="30" t="inlineStr">
+        <is>
+          <t>[Corregido 24/10] RoleManagementServiceTest (7 tests). La cuenta PLATFORM_ADMIN se activa por ENV_FILE (plantilla en docs/despliegue-vps.md). e2e.sh recorre el criterio completo: rol nuevo → permisos → usuario → acceso permitido y 403 donde corresponde.
+[Revisión de código 23/10] API de roles implementada (crear, editar, desactivar, permisos, roles asignables, incompatibilidades). Falta: tests automatizados (solo hay colección Postman) y una cuenta PLATFORM_ADMIN para la demo: solo ese rol tiene identity.role.manage y no existe por defecto (PLATFORM_ADMIN_SEED_ENABLED=false).</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="25" t="inlineStr">
@@ -3444,7 +3495,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M20" s="14" t="n">
+      <c r="M20" s="48" t="n">
         <v>6</v>
       </c>
       <c r="N20" s="12" t="inlineStr">
@@ -3474,10 +3525,14 @@
       </c>
       <c r="S20" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T20" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T20" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] No queda ningún @RequiresRole; el gateway propaga X-Permissions desde el JWT y descarta los que envía el cliente. Tests del interceptor.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="25" t="inlineStr">
@@ -3538,7 +3593,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M21" s="14" t="n">
+      <c r="M21" s="48" t="n">
         <v>5</v>
       </c>
       <c r="N21" s="12" t="inlineStr">
@@ -3568,10 +3623,14 @@
       </c>
       <c r="S21" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T21" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T21" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] Denegar por defecto: todos los endpoints declaran su control (check_permissions.py); sin token responde 401.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="25" t="inlineStr">
@@ -3632,7 +3691,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M22" s="14" t="n">
+      <c r="M22" s="48" t="n">
         <v>5</v>
       </c>
       <c r="N22" s="12" t="inlineStr">
@@ -3662,10 +3721,15 @@
       </c>
       <c r="S22" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T22" s="30" t="inlineStr"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="T22" s="30" t="inlineStr">
+        <is>
+          <t>[Corregido 24/10] Desbloqueada: con la cuenta PLATFORM_ADMIN la matriz se puede editar. Falta solo recorrer la demo en vivo desde la pantalla.
+[Frontend 24/10] Pantallas de roles y matriz (169 permisos × 6 roles) con exportación CSV/Excel, verificadas en el navegador. Para la demo de editar la matriz hace falta una cuenta PLATFORM_ADMIN (mismo bloqueo que RBAC-02): ADMINISTRATOR no tiene identity.role.manage.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="25" t="inlineStr">
@@ -3726,7 +3790,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M23" s="14" t="n">
+      <c r="M23" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N23" s="12" t="inlineStr">
@@ -3820,7 +3884,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M24" s="14" t="n">
+      <c r="M24" s="48" t="n">
         <v>4</v>
       </c>
       <c r="N24" s="12" t="inlineStr">
@@ -3850,10 +3914,14 @@
       </c>
       <c r="S24" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T24" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T24" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] Reportes Trivy (fs e imágenes) y ZAP del 12/10 en docs/seguridad/escaneos/antes/.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="25" t="inlineStr">
@@ -3914,7 +3982,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M25" s="14" t="n">
+      <c r="M25" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N25" s="12" t="inlineStr">
@@ -3944,10 +4012,14 @@
       </c>
       <c r="S25" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T25" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T25" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] Solo el gateway (8080) y Keycloak (18080) publican puerto; X-User-Id/X-Roles falsos sin token → 401 (e2e.sh).</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="25" t="inlineStr">
@@ -4008,7 +4080,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M26" s="14" t="n">
+      <c r="M26" s="48" t="n">
         <v>4</v>
       </c>
       <c r="N26" s="12" t="inlineStr">
@@ -4038,10 +4110,14 @@
       </c>
       <c r="S26" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T26" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T26" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] Probado: tras el logout, el mismo token recibe 401 en pacientes, historial y facturación.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
@@ -4102,7 +4178,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="M27" s="48" t="n">
         <v>2</v>
       </c>
       <c r="N27" s="12" t="inlineStr">
@@ -4132,10 +4208,16 @@
       </c>
       <c r="S27" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T27" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T27" s="30" t="inlineStr">
+        <is>
+          <t>[Corregido 24/10] La contraseña demo ya no está en el código del frontend: el botón de cuenta demo completa solo el correo.
+[Revisión de código 23/10] Webhook sin firma → 401; con meta y sin WHATSAPP_APP_SECRET no arranca; CORS por lista exacta (origen ajeno → 403); cuentas demo apagadas; /internal de identidad denyAll; actuator sin detalles. Ojo: el .env local de Nicole tiene GATEWAY_ALLOWED_ORIGINS=*.
+[Frontend 24/10] Observación: el frontend tiene DEMO_PASSWORD = 'Demo1234!' en login-page.ts, que viaja en el JavaScript público. Además ya no coincide con la contraseña demo por defecto del backend (SanGabriel.Demo26!).</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="25" t="inlineStr">
@@ -4196,7 +4278,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="M28" s="48" t="n">
         <v>4</v>
       </c>
       <c r="N28" s="12" t="inlineStr">
@@ -4226,10 +4308,16 @@
       </c>
       <c r="S28" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T28" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T28" s="30" t="inlineStr">
+        <is>
+          <t>[Corregido 24/10] Frontend: nginx con CSP (script-src 'self'), X-Frame-Options, nosniff, Referrer-Policy y Permissions-Policy, sin versión en Server; Caddy agrega HSTS. Verificado en el navegador: sin violaciones de CSP.
+[Revisión de código 23/10] Cabeceras HSTS, nosniff, X-Frame-Options, CSP y Referrer-Policy verificadas; re-escaneo del 12/10 con 0 críticas y 0 altas.
+[Frontend 24/10] Falta en el frontend: nginx sirve el HTML y el JS sin cabeceras de seguridad (CSP, X-Frame-Options, nosniff, Referrer-Policy, HSTS) y expone su versión (Server: nginx/1.27.5). Las dependencias del frontend quedaron en 0 vulnerabilidades (Angular 22.2.3).</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="25" t="inlineStr">
@@ -4290,7 +4378,7 @@
           <t>Baja</t>
         </is>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="M29" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N29" s="12" t="inlineStr">
@@ -4320,10 +4408,14 @@
       </c>
       <c r="S29" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T29" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T29" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] Con MySQL local cada servicio tiene su usuario: marketing_user no puede leer identity_db (probado).</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="25" t="inlineStr">
@@ -4384,7 +4476,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="M30" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N30" s="12" t="inlineStr">
@@ -4414,10 +4506,14 @@
       </c>
       <c r="S30" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T30" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T30" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] Comparativa en docs/seguridad/escaneos/despues/. Recomendado: re-escanear la versión final, porque Keycloak 26.7.5, IAM y LOG se integraron después del 12/10.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="25" t="inlineStr">
@@ -4478,7 +4574,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M31" s="14" t="n">
+      <c r="M31" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N31" s="12" t="inlineStr">
@@ -4508,10 +4604,14 @@
       </c>
       <c r="S31" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T31" s="30" t="inlineStr"/>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="T31" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] El servicio cloudflared está listo en compose (perfil publico), pero no hay token configurado ni URL pública confirmada; el deploy al VPS está pausado.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="25" t="inlineStr">
@@ -4572,7 +4672,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M32" s="14" t="n">
+      <c r="M32" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N32" s="12" t="inlineStr">
@@ -4666,7 +4766,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M33" s="14" t="n">
+      <c r="M33" s="48" t="n">
         <v>4</v>
       </c>
       <c r="N33" s="12" t="inlineStr">
@@ -4696,10 +4796,14 @@
       </c>
       <c r="S33" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T33" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T33" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] La descarga se bloquea con 409 INTEGRITY_MISMATCH y evento de auditoría; GET /documents/{id}/integrity (permiso documents.document.read); cubre los consentimientos firmados. Tests.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="25" t="inlineStr">
@@ -4760,7 +4864,7 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="M34" s="14" t="n">
+      <c r="M34" s="48" t="n">
         <v>2</v>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -4790,10 +4894,14 @@
       </c>
       <c r="S34" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T34" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T34" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] scripts/checksums.sh y checksums.ps1 con SHA-256 y comparación con CRC32 y MD5.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="25" t="inlineStr">
@@ -4854,7 +4962,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M35" s="14" t="n">
+      <c r="M35" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N35" s="12" t="inlineStr">
@@ -4948,7 +5056,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="M36" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N36" s="12" t="inlineStr">
@@ -4978,10 +5086,16 @@
       </c>
       <c r="S36" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T36" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T36" s="30" t="inlineStr">
+        <is>
+          <t>[Corregido 24/10] La IP guardada es la del usuario: el gateway la calcula (solo cree X-Forwarded-For de un proxy interno) y la pasa en X-Client-Ip, que descarta si la manda el cliente. Verificado en e2e.sh.
+[Revisión de código 23/10] LOGIN_SUCCESS, LOGIN_FAILED, ACCOUNT_LOCKED y LOGOUT llegan a audit_db; cadena de hash íntegra (155 eventos). Corregido el 23/10: los intentos fallidos y con correos inexistentes se perdían.
+[Frontend 24/10] Observación: la IP que se guarda es la del gateway (172.19.x.x), no la del usuario: AuditTrail usa request.getRemoteAddr() y nadie lee X-Forwarded-For.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="25" t="inlineStr">
@@ -5042,7 +5156,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M37" s="14" t="n">
+      <c r="M37" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N37" s="12" t="inlineStr">
@@ -5072,10 +5186,15 @@
       </c>
       <c r="S37" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T37" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T37" s="30" t="inlineStr">
+        <is>
+          <t>[Corregido 24/10] Ahora también se auditan los roles (ROLE_CREATED/UPDATED/DISABLED/PERMISSIONS_CHANGED/ASSIGNABLE_ROLES_CHANGED/INCOMPATIBILITY_*) y los 403 de todos los servicios, que registra el gateway como ACCESS_DENIED. Verificado en e2e.sh.
+[Revisión de código 23/10] Verificado en la bitácora: USER_CREATED/UPDATED/DISABLED, ACCOUNT_LOCKED/UNLOCKED, PASSWORD_RESET/CHANGED. Implementado sin prueba en vivo: ROLE_ASSIGNED/REVOKED y ACCESS_DENIED de identidad. Falta: ROLE_CREATED/DISABLED/PERMISSIONS_CHANGED (RoleManagementService no audita) y ACCESS_DENIED en los interceptores de los demás servicios.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="25" t="inlineStr">
@@ -5136,7 +5255,7 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="M38" s="14" t="n">
+      <c r="M38" s="48" t="n">
         <v>2</v>
       </c>
       <c r="N38" s="12" t="inlineStr">
@@ -5166,10 +5285,15 @@
       </c>
       <c r="S38" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T38" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T38" s="30" t="inlineStr">
+        <is>
+          <t>[Corregido 24/10] ms-gateway con logback estructurado y correlation id en el MDC: los 14 servicios con el mismo formato.
+[Revisión de código 23/10] Logback estructurado con correlation id en 13 de 14 servicios: falta ms-gateway. Una muestra de logs del flujo completo no contiene tokens ni contraseñas.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="25" t="inlineStr">
@@ -5230,7 +5354,7 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="M39" s="14" t="n">
+      <c r="M39" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N39" s="12" t="inlineStr">
@@ -5260,10 +5384,14 @@
       </c>
       <c r="S39" s="29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="T39" s="30" t="inlineStr"/>
+          <t>Hecha</t>
+        </is>
+      </c>
+      <c r="T39" s="30" t="inlineStr">
+        <is>
+          <t>[Frontend 24/10] Pantalla de bitácora verificada en el navegador: cadena íntegra (158 eventos), resumen, filtros por área/resultado/acción, columna IP, exportación CSV y botón Verificar integridad. Solo ve la ruta quien tiene el permiso.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="25" t="inlineStr">
@@ -5324,7 +5452,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M40" s="14" t="n">
+      <c r="M40" s="48" t="n">
         <v>1</v>
       </c>
       <c r="N40" s="12" t="inlineStr">
@@ -5418,7 +5546,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M41" s="14" t="n">
+      <c r="M41" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N41" s="12" t="inlineStr">
@@ -5512,7 +5640,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M42" s="14" t="n">
+      <c r="M42" s="48" t="n">
         <v>2</v>
       </c>
       <c r="N42" s="12" t="inlineStr">
@@ -5606,7 +5734,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M43" s="14" t="n">
+      <c r="M43" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N43" s="12" t="inlineStr">
@@ -5700,7 +5828,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M44" s="14" t="n">
+      <c r="M44" s="48" t="n">
         <v>7</v>
       </c>
       <c r="N44" s="12" t="inlineStr">
@@ -5794,7 +5922,7 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="M45" s="14" t="n">
+      <c r="M45" s="48" t="n">
         <v>4</v>
       </c>
       <c r="N45" s="12" t="inlineStr">
@@ -5888,7 +6016,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M46" s="14" t="n">
+      <c r="M46" s="48" t="n">
         <v>5</v>
       </c>
       <c r="N46" s="12" t="inlineStr">
@@ -5982,7 +6110,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M47" s="14" t="n">
+      <c r="M47" s="48" t="n">
         <v>4</v>
       </c>
       <c r="N47" s="12" t="inlineStr">
@@ -6076,7 +6204,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M48" s="14" t="n">
+      <c r="M48" s="48" t="n">
         <v>6</v>
       </c>
       <c r="N48" s="12" t="inlineStr">
@@ -6109,7 +6237,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="T48" s="30" t="inlineStr"/>
+      <c r="T48" s="30" t="inlineStr">
+        <is>
+          <t>[Revisión de código 23/10] Módulo fuera del sistema y de este repo: no se puede verificar aquí.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="25" t="inlineStr">
@@ -6170,7 +6302,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M49" s="14" t="n">
+      <c r="M49" s="48" t="n">
         <v>2</v>
       </c>
       <c r="N49" s="12" t="inlineStr">
@@ -6264,7 +6396,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M50" s="14" t="n">
+      <c r="M50" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="N50" s="12" t="inlineStr">
@@ -6358,7 +6490,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M51" s="14" t="n">
+      <c r="M51" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="N51" s="12" t="inlineStr">
@@ -6452,7 +6584,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M52" s="14" t="n">
+      <c r="M52" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="N52" s="12" t="inlineStr">
@@ -6546,7 +6678,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M53" s="14" t="n">
+      <c r="M53" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="N53" s="12" t="inlineStr">
@@ -6640,7 +6772,7 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="M54" s="14" t="n">
+      <c r="M54" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="N54" s="12" t="inlineStr">
@@ -6734,7 +6866,7 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="M55" s="14" t="n">
+      <c r="M55" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="N55" s="12" t="inlineStr">
@@ -6828,7 +6960,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M56" s="14" t="n">
+      <c r="M56" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="N56" s="12" t="inlineStr">
@@ -6922,7 +7054,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M57" s="14" t="n">
+      <c r="M57" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="N57" s="12" t="inlineStr">
@@ -7016,7 +7148,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M58" s="14" t="n">
+      <c r="M58" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="N58" s="12" t="inlineStr">
@@ -7110,7 +7242,7 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="M59" s="14" t="n">
+      <c r="M59" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="N59" s="12" t="inlineStr">
@@ -7204,7 +7336,7 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="M60" s="14" t="n">
+      <c r="M60" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="N60" s="12" t="inlineStr">
@@ -7298,7 +7430,7 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="M61" s="14" t="n">
+      <c r="M61" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="N61" s="12" t="inlineStr">
@@ -7392,7 +7524,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M62" s="14" t="n">
+      <c r="M62" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="N62" s="12" t="inlineStr">
@@ -7486,7 +7618,7 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="M63" s="14" t="n">
+      <c r="M63" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="N63" s="12" t="inlineStr">
@@ -7580,7 +7712,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M64" s="14" t="n">
+      <c r="M64" s="48" t="n">
         <v>1</v>
       </c>
       <c r="N64" s="12" t="inlineStr">
@@ -7674,7 +7806,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M65" s="14" t="n">
+      <c r="M65" s="48" t="n">
         <v>4</v>
       </c>
       <c r="N65" s="12" t="inlineStr">
@@ -7768,7 +7900,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M66" s="14" t="n">
+      <c r="M66" s="48" t="n">
         <v>2</v>
       </c>
       <c r="N66" s="12" t="inlineStr">
@@ -7862,7 +7994,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M67" s="14" t="n">
+      <c r="M67" s="48" t="n">
         <v>2</v>
       </c>
       <c r="N67" s="12" t="inlineStr">
@@ -7956,7 +8088,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M68" s="14" t="n">
+      <c r="M68" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="N68" s="12" t="inlineStr">
@@ -8050,7 +8182,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M69" s="14" t="n">
+      <c r="M69" s="48" t="n">
         <v>2</v>
       </c>
       <c r="N69" s="12" t="inlineStr">
@@ -8144,7 +8276,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M70" s="14" t="n">
+      <c r="M70" s="48" t="n">
         <v>2</v>
       </c>
       <c r="N70" s="12" t="inlineStr">
@@ -8238,7 +8370,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M71" s="14" t="n">
+      <c r="M71" s="48" t="n">
         <v>1.5</v>
       </c>
       <c r="N71" s="12" t="inlineStr">
@@ -8332,7 +8464,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M72" s="14" t="n">
+      <c r="M72" s="48" t="n">
         <v>2</v>
       </c>
       <c r="N72" s="12" t="inlineStr">
@@ -8426,7 +8558,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M73" s="14" t="n">
+      <c r="M73" s="48" t="n">
         <v>4</v>
       </c>
       <c r="N73" s="12" t="inlineStr">
@@ -8520,7 +8652,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="M74" s="14" t="n">
+      <c r="M74" s="48" t="n">
         <v>4</v>
       </c>
       <c r="N74" s="12" t="inlineStr">
@@ -8614,7 +8746,7 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="M75" s="14" t="n">
+      <c r="M75" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N75" s="12" t="inlineStr">
@@ -8708,7 +8840,7 @@
           <t>Urgente</t>
         </is>
       </c>
-      <c r="M76" s="14" t="n">
+      <c r="M76" s="48" t="n">
         <v>0.5</v>
       </c>
       <c r="N76" s="12" t="inlineStr">
@@ -8802,7 +8934,7 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="M77" s="14" t="n">
+      <c r="M77" s="48" t="n">
         <v>3</v>
       </c>
       <c r="N77" s="12" t="inlineStr">
@@ -9060,39 +9192,39 @@
           <t>Nicole</t>
         </is>
       </c>
-      <c r="B5" s="14">
+      <c r="B5" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A5,Tareas!$I$5:$I$77,B$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="C5" s="14">
+      <c r="C5" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A5,Tareas!$I$5:$I$77,C$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A5,Tareas!$I$5:$I$77,D$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="E5" s="14">
+      <c r="E5" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A5,Tareas!$I$5:$I$77,E$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="F5" s="14">
+      <c r="F5" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A5,Tareas!$I$5:$I$77,F$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="G5" s="14">
+      <c r="G5" s="48">
         <f>SUM(B5:F5)</f>
         <v/>
       </c>
-      <c r="H5" s="14">
+      <c r="H5" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A5,Tareas!$L$5:$L$77,"Baja")</f>
         <v/>
       </c>
-      <c r="I5" s="14">
+      <c r="I5" s="48">
         <f>COUNTIF(Tareas!$D$5:$D$77,$A5)</f>
         <v/>
       </c>
-      <c r="J5" s="14">
+      <c r="J5" s="48">
         <f>COUNTIFS(Tareas!$D$5:$D$77,$A5,Tareas!$S$5:$S$77,"Hecha")</f>
         <v/>
       </c>
@@ -9107,39 +9239,39 @@
           <t>Franco</t>
         </is>
       </c>
-      <c r="B6" s="14">
+      <c r="B6" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A6,Tareas!$I$5:$I$77,B$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="C6" s="14">
+      <c r="C6" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A6,Tareas!$I$5:$I$77,C$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A6,Tareas!$I$5:$I$77,D$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="E6" s="14">
+      <c r="E6" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A6,Tareas!$I$5:$I$77,E$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="F6" s="14">
+      <c r="F6" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A6,Tareas!$I$5:$I$77,F$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="G6" s="14">
+      <c r="G6" s="48">
         <f>SUM(B6:F6)</f>
         <v/>
       </c>
-      <c r="H6" s="14">
+      <c r="H6" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A6,Tareas!$L$5:$L$77,"Baja")</f>
         <v/>
       </c>
-      <c r="I6" s="14">
+      <c r="I6" s="48">
         <f>COUNTIF(Tareas!$D$5:$D$77,$A6)</f>
         <v/>
       </c>
-      <c r="J6" s="14">
+      <c r="J6" s="48">
         <f>COUNTIFS(Tareas!$D$5:$D$77,$A6,Tareas!$S$5:$S$77,"Hecha")</f>
         <v/>
       </c>
@@ -9154,39 +9286,39 @@
           <t>Juanjo</t>
         </is>
       </c>
-      <c r="B7" s="14">
+      <c r="B7" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A7,Tareas!$I$5:$I$77,B$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A7,Tareas!$I$5:$I$77,C$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A7,Tareas!$I$5:$I$77,D$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A7,Tareas!$I$5:$I$77,E$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="F7" s="14">
+      <c r="F7" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A7,Tareas!$I$5:$I$77,F$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="G7" s="14">
+      <c r="G7" s="48">
         <f>SUM(B7:F7)</f>
         <v/>
       </c>
-      <c r="H7" s="14">
+      <c r="H7" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A7,Tareas!$L$5:$L$77,"Baja")</f>
         <v/>
       </c>
-      <c r="I7" s="14">
+      <c r="I7" s="48">
         <f>COUNTIF(Tareas!$D$5:$D$77,$A7)</f>
         <v/>
       </c>
-      <c r="J7" s="14">
+      <c r="J7" s="48">
         <f>COUNTIFS(Tareas!$D$5:$D$77,$A7,Tareas!$S$5:$S$77,"Hecha")</f>
         <v/>
       </c>
@@ -9201,39 +9333,39 @@
           <t>Alvaro</t>
         </is>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A8,Tareas!$I$5:$I$77,B$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A8,Tareas!$I$5:$I$77,C$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A8,Tareas!$I$5:$I$77,D$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A8,Tareas!$I$5:$I$77,E$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="F8" s="14">
+      <c r="F8" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A8,Tareas!$I$5:$I$77,F$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="G8" s="14">
+      <c r="G8" s="48">
         <f>SUM(B8:F8)</f>
         <v/>
       </c>
-      <c r="H8" s="14">
+      <c r="H8" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A8,Tareas!$L$5:$L$77,"Baja")</f>
         <v/>
       </c>
-      <c r="I8" s="14">
+      <c r="I8" s="48">
         <f>COUNTIF(Tareas!$D$5:$D$77,$A8)</f>
         <v/>
       </c>
-      <c r="J8" s="14">
+      <c r="J8" s="48">
         <f>COUNTIFS(Tareas!$D$5:$D$77,$A8,Tareas!$S$5:$S$77,"Hecha")</f>
         <v/>
       </c>
@@ -9248,39 +9380,39 @@
           <t>Alan</t>
         </is>
       </c>
-      <c r="B9" s="14">
+      <c r="B9" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A9,Tareas!$I$5:$I$77,B$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A9,Tareas!$I$5:$I$77,C$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A9,Tareas!$I$5:$I$77,D$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="E9" s="14">
+      <c r="E9" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A9,Tareas!$I$5:$I$77,E$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="F9" s="14">
+      <c r="F9" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A9,Tareas!$I$5:$I$77,F$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="G9" s="14">
+      <c r="G9" s="48">
         <f>SUM(B9:F9)</f>
         <v/>
       </c>
-      <c r="H9" s="14">
+      <c r="H9" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A9,Tareas!$L$5:$L$77,"Baja")</f>
         <v/>
       </c>
-      <c r="I9" s="14">
+      <c r="I9" s="48">
         <f>COUNTIF(Tareas!$D$5:$D$77,$A9)</f>
         <v/>
       </c>
-      <c r="J9" s="14">
+      <c r="J9" s="48">
         <f>COUNTIFS(Tareas!$D$5:$D$77,$A9,Tareas!$S$5:$S$77,"Hecha")</f>
         <v/>
       </c>
@@ -9295,39 +9427,39 @@
           <t>Favian</t>
         </is>
       </c>
-      <c r="B10" s="14">
+      <c r="B10" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A10,Tareas!$I$5:$I$77,B$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A10,Tareas!$I$5:$I$77,C$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A10,Tareas!$I$5:$I$77,D$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A10,Tareas!$I$5:$I$77,E$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="F10" s="14">
+      <c r="F10" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A10,Tareas!$I$5:$I$77,F$4,Tareas!$L$5:$L$77,"&lt;&gt;Baja")</f>
         <v/>
       </c>
-      <c r="G10" s="14">
+      <c r="G10" s="48">
         <f>SUM(B10:F10)</f>
         <v/>
       </c>
-      <c r="H10" s="14">
+      <c r="H10" s="48">
         <f>SUMIFS(Tareas!$M$5:$M$77,Tareas!$D$5:$D$77,$A10,Tareas!$L$5:$L$77,"Baja")</f>
         <v/>
       </c>
-      <c r="I10" s="14">
+      <c r="I10" s="48">
         <f>COUNTIF(Tareas!$D$5:$D$77,$A10)</f>
         <v/>
       </c>
-      <c r="J10" s="14">
+      <c r="J10" s="48">
         <f>COUNTIFS(Tareas!$D$5:$D$77,$A10,Tareas!$S$5:$S$77,"Hecha")</f>
         <v/>
       </c>
@@ -9342,39 +9474,39 @@
           <t>Equipo</t>
         </is>
       </c>
-      <c r="B11" s="36">
+      <c r="B11" s="49">
         <f>SUM(B5:B10)</f>
         <v/>
       </c>
-      <c r="C11" s="36">
+      <c r="C11" s="49">
         <f>SUM(C5:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="36">
+      <c r="D11" s="49">
         <f>SUM(D5:D10)</f>
         <v/>
       </c>
-      <c r="E11" s="36">
+      <c r="E11" s="49">
         <f>SUM(E5:E10)</f>
         <v/>
       </c>
-      <c r="F11" s="36">
+      <c r="F11" s="49">
         <f>SUM(F5:F10)</f>
         <v/>
       </c>
-      <c r="G11" s="36">
+      <c r="G11" s="49">
         <f>SUM(G5:G10)</f>
         <v/>
       </c>
-      <c r="H11" s="36">
+      <c r="H11" s="49">
         <f>SUM(H5:H10)</f>
         <v/>
       </c>
-      <c r="I11" s="36">
+      <c r="I11" s="49">
         <f>SUM(I5:I10)</f>
         <v/>
       </c>
-      <c r="J11" s="36">
+      <c r="J11" s="49">
         <f>SUM(J5:J10)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Guia del VPS y plan del sprint: la gestion de roles es del OSI desde ISO-01
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etica docs/Plan_Sprint_SIS321_MedicalSys.xlsx
+++ b/etica docs/Plan_Sprint_SIS321_MedicalSys.xlsx
@@ -1793,8 +1793,8 @@
     <mergeCell ref="B43:H43"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B50:G50"/>
+    <mergeCell ref="A5:H5"/>
     <mergeCell ref="B42:H42"/>
-    <mergeCell ref="A5:H5"/>
     <mergeCell ref="C34:H34"/>
     <mergeCell ref="B60:H60"/>
     <mergeCell ref="C30:H30"/>
@@ -3431,7 +3431,8 @@
       </c>
       <c r="T19" s="30" t="inlineStr">
         <is>
-          <t>[Corregido 24/10] RoleManagementServiceTest (7 tests). La cuenta PLATFORM_ADMIN se activa por ENV_FILE (plantilla en docs/despliegue-vps.md). e2e.sh recorre el criterio completo: rol nuevo → permisos → usuario → acceso permitido y 403 donde corresponde.
+          <t>[Actualizado 24/10, ISO-01] Desde la migración V9 de Alvaro, la gestión de roles y permisos es del OSI (ya no de PLATFORM_ADMIN). e2e.sh recorre el criterio con la cuenta OSI: rol nuevo → permiso → cuenta → nivel MAC → acceso, y el 403 donde corresponde.
+[Corregido 24/10] RoleManagementServiceTest (7 tests). La cuenta PLATFORM_ADMIN se activa por ENV_FILE (plantilla en docs/despliegue-vps.md). e2e.sh recorre el criterio completo: rol nuevo → permisos → usuario → acceso permitido y 403 donde corresponde.
 [Revisión de código 23/10] API de roles implementada (crear, editar, desactivar, permisos, roles asignables, incompatibilidades). Falta: tests automatizados (solo hay colección Postman) y una cuenta PLATFORM_ADMIN para la demo: solo ese rol tiene identity.role.manage y no existe por defecto (PLATFORM_ADMIN_SEED_ENABLED=false).</t>
         </is>
       </c>
@@ -3726,7 +3727,8 @@
       </c>
       <c r="T22" s="30" t="inlineStr">
         <is>
-          <t>[Corregido 24/10] Desbloqueada: con la cuenta PLATFORM_ADMIN la matriz se puede editar. Falta solo recorrer la demo en vivo desde la pantalla.
+          <t>[Actualizado 24/10, ISO-01] La matriz se edita con la cuenta OSI (OSI_SEED_ENABLED en ENV_FILE). Falta en el frontend una pantalla para fijar el nivel MAC de una cuenta: hoy solo por API (PUT /users/{id}/clearance).
+[Corregido 24/10] Desbloqueada: con la cuenta PLATFORM_ADMIN la matriz se puede editar. Falta solo recorrer la demo en vivo desde la pantalla.
 [Frontend 24/10] Pantallas de roles y matriz (169 permisos × 6 roles) con exportación CSV/Excel, verificadas en el navegador. Para la demo de editar la matriz hace falta una cuenta PLATFORM_ADMIN (mismo bloqueo que RBAC-02): ADMINISTRATOR no tiene identity.role.manage.</t>
         </is>
       </c>

</xml_diff>